<commit_message>
feat(sales): enable full sales bill editing with coordinated PDF, QR, and registers
</commit_message>
<xml_diff>
--- a/test-exports/cashbook-2020-01-01-to-2030-01-01.xlsx
+++ b/test-exports/cashbook-2020-01-01-to-2030-01-01.xlsx
@@ -344,196 +344,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="KusumExport1" displayName="KusumExport1" ref="A6:L16" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A6:L16">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="12">
-    <tableColumn id="1" name="Date" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Type" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Payment method" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Description" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Money in" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Money out" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Running balance" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Reference" totalsRowFunction="none"/>
-    <tableColumn id="9" name="Customer phone" totalsRowFunction="none"/>
-    <tableColumn id="10" name="Customer" totalsRowFunction="none"/>
-    <tableColumn id="11" name="Ledger synced" totalsRowFunction="none"/>
-    <tableColumn id="12" name="Notes" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" name="KusumExport2" displayName="KusumExport2" ref="A6:E10" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A6:E10">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Payment method" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Total entries" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Total money in" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Total money out" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Net balance" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" name="KusumExport3" displayName="KusumExport3" ref="A6:L9" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A6:L9">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="12">
-    <tableColumn id="1" name="Date" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Type" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Payment method" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Description" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Money in" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Money out" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Running balance" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Reference" totalsRowFunction="none"/>
-    <tableColumn id="9" name="Customer phone" totalsRowFunction="none"/>
-    <tableColumn id="10" name="Customer" totalsRowFunction="none"/>
-    <tableColumn id="11" name="Ledger synced" totalsRowFunction="none"/>
-    <tableColumn id="12" name="Notes" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" name="KusumExport4" displayName="KusumExport4" ref="A6:L9" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A6:L9">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="12">
-    <tableColumn id="1" name="Date" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Type" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Payment method" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Description" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Money in" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Money out" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Running balance" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Reference" totalsRowFunction="none"/>
-    <tableColumn id="9" name="Customer phone" totalsRowFunction="none"/>
-    <tableColumn id="10" name="Customer" totalsRowFunction="none"/>
-    <tableColumn id="11" name="Ledger synced" totalsRowFunction="none"/>
-    <tableColumn id="12" name="Notes" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" name="KusumExport5" displayName="KusumExport5" ref="A6:L7" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A6:L7">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="12">
-    <tableColumn id="1" name="Date" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Type" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Payment method" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Description" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Money in" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Money out" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Running balance" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Reference" totalsRowFunction="none"/>
-    <tableColumn id="9" name="Customer phone" totalsRowFunction="none"/>
-    <tableColumn id="10" name="Customer" totalsRowFunction="none"/>
-    <tableColumn id="11" name="Ledger synced" totalsRowFunction="none"/>
-    <tableColumn id="12" name="Notes" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" name="KusumExport6" displayName="KusumExport6" ref="A6:L9" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A6:L9">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="12">
-    <tableColumn id="1" name="Date" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Type" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Payment method" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Description" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Money in" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Money out" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Running balance" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Reference" totalsRowFunction="none"/>
-    <tableColumn id="9" name="Customer phone" totalsRowFunction="none"/>
-    <tableColumn id="10" name="Customer" totalsRowFunction="none"/>
-    <tableColumn id="11" name="Ledger synced" totalsRowFunction="none"/>
-    <tableColumn id="12" name="Notes" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1325,9 +1135,6 @@
     <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
   </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1487,9 +1294,6 @@
     <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
   </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1734,9 +1538,6 @@
     <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
   </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1981,9 +1782,6 @@
     <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
   </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2168,9 +1966,6 @@
     <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
   </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2415,8 +2210,5 @@
     <oddFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenFooter>&amp;LKusum ERP&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
   </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>